<commit_message>
docs: 지점당 등록 회원 가정 550명 → 약 280명(하루 100명 × 7 ÷ 주 2.5회) (D40, log/070)
design-constants ②를 ③(하루 이용자 100명)에서 역산하도록 바꿔 두 가정을 맞췄다.
전사 회원 수 추정: 지금 ≈2.3만, 3년 후 ≈3.1만(이전 ≈6만). 회원관리·인사정보관리·
traffic-infra-review 갱신, 요구사항 정의서 재생성. 하루 요청 수·피크 rps는 변화 없음.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CARwBkVUSFMnxCdPq1HrjQ
</commit_message>
<xml_diff>
--- a/docs/deliverables/요구사항정의서.xlsx
+++ b/docs/deliverables/요구사항정의서.xlsx
@@ -242,7 +242,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286 — </t>
+      <t xml:space="preserve">b4f9e1e — </t>
     </r>
     <r>
       <rPr>
@@ -16227,7 +16227,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>
@@ -17333,7 +17333,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>
@@ -18312,7 +18312,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>
@@ -18966,7 +18966,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>
@@ -19359,7 +19359,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>
@@ -19986,7 +19986,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>
@@ -20767,7 +20767,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>
@@ -21341,7 +21341,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>
@@ -21786,7 +21786,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">8fce286)</t>
+      <t xml:space="preserve">b4f9e1e)</t>
     </r>
   </si>
   <si>

</xml_diff>

<commit_message>
docs+fix: RFP 보안 문서 셋과 문서 주소 XSS 수정(log/139, D53)
- 보안관리계획(N8-1): 인원·문서·장비·비밀값·위탁, 지금 약점 9건과 조치 계획
- 개발보안 점검표(N2-1): 행안부 구현단계 보안약점 49개 — 대응 34·부분 4·해당 없음 11
- 의존성 라이선스(N10): scripts/license-report.mjs, 운영 의존성 219개 모두 허용형
- 점검 중 발견(입력-4 XSS): 문서 fileUrl을 http(s)만 받고 화면도 http(s)만 링크로,
  document-rules.spec.ts에 javascript:·data:·상대 경로 400 케이스
- 요구사항추적표 §3 집계 73% → 80%, 요구사항 정의서 재생성

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhHabvYheW2oxJWYuUifjJ
</commit_message>
<xml_diff>
--- a/docs/deliverables/요구사항정의서.xlsx
+++ b/docs/deliverables/요구사항정의서.xlsx
@@ -24,7 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="범위 제외" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'요구사항 총괄'!$A$11:$G$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'요구사항 총괄'!$A$11:$G$182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RFP 충족 판정'!$A$17:$E$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -659,7 +659,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>도메인 9개 · 기능(API) 97개 · 불변규칙 26개 · RFP 미구현·부분 9건 · 자동 테스트 파일 43개</t>
+          <t>도메인 9개 · 기능(API) 97개 · 불변규칙 26개 · RFP 미구현·부분 6건 · 자동 테스트 파일 43개</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>조항 72개 중 해당 없음 8개를 뺀 충족률 47/64 = 73% / 94%(구현+조정 / 부분 포함)</t>
+          <t>조항 72개 중 해당 없음 8개를 뺀 충족률 51/64 = 80% / 95%(구현+조정 / 부분 포함)</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4030,17 +4030,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>설치및운영(1-2 #2)</t>
+          <t>과업4·산출물5(p.4·p.7)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>소프트웨어 개발보안 준수</t>
+          <t>이용자 매뉴얼 제작·게시판 탑재, 어플 사용 교육 자료</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>부분 — 개별 조치는 있지만(§1-2 #2) 시큐어코딩 점검 기준표·점검 기록이 없다</t>
+          <t>부분 — 관리자 웹 화면별 도움말과 회원 웹 이용 안내는 있다. 별도 사용자 매뉴얼(교육 자료 1편)과 게시판 탑재는 없다. 대면 교육은 해당 없음</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -4057,129 +4057,48 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>보안요건(1-2 #8)</t>
+          <t>산출물4(p.7)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>보안관리계획(인원·문서·장비)</t>
+          <t>단계별 개발 진행 보고서 5부</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>없다. 개인정보처리방침은 회원 웹 초안으로 작성(D51)</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>미구현</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>GAP-07</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>규정의준수(1-2 #10)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>지식재산권·저작권 점검</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>부분 — 오픈소스만 쓰지만 의존성 라이선스 목록·점검 기록이 없다</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
+          <t>부분 — 진행 기록(docs/log/ 130여 건)·발표 자료는 있지만 개발·테스트·검수·도입·기대효과 단계별 보고서 형식은 없다</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>부분</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>GAP-08</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>과업4·산출물5(p.4·p.7)</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>이용자 매뉴얼 제작·게시판 탑재, 어플 사용 교육 자료</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>부분 — 관리자 웹 화면별 도움말과 회원 웹 이용 안내는 있다. 별도 사용자 매뉴얼(교육 자료 1편)과 게시판 탑재는 없다. 대면 교육은 해당 없음</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>GAP-09</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>산출물4(p.7)</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>단계별 개발 진행 보고서 5부</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>부분 — 진행 기록(docs/log/ 130여 건)·발표 자료는 있지만 개발·테스트·검수·도입·기대효과 단계별 보고서 형식은 없다</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>API는 있고 화면이 없는 것</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>지금은 없다(로컬 전용 dev-storage 경로 제외). 마지막 항목이던 관리자의 직원 업무일지 열람은 2026-10-14 직원 상세에 붙였다(D51, log/112).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>API는 있고 화면이 없는 것</t>
+          <t>설계는 있지만 미구현인 도메인 규칙</t>
         </is>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1">
       <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>지금은 없다(로컬 전용 dev-storage 경로 제외). 마지막 항목이던 관리자의 직원 업무일지 열람은 2026-10-14 직원 상세에 붙였다(D51, log/112).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>설계는 있지만 미구현인 도메인 규칙</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>결제 PaymentGateway 어댑터(ADR-RSV-03) — 실 PG를 붙일 때 필요하다.</t>
         </is>
@@ -4188,7 +4107,7 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A13:E13"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4386,7 +4305,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G185"/>
+  <dimension ref="A1:G182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4431,7 +4350,7 @@
         </is>
       </c>
       <c r="B5" s="8">
-        <f>COUNTIF($C$12:$C$186,"기능")</f>
+        <f>COUNTIF($C$12:$C$183,"기능")</f>
         <v/>
       </c>
     </row>
@@ -4442,7 +4361,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>COUNTIFS($C$12:$C$186,"기능",$F$12:$F$186,"있음")</f>
+        <f>COUNTIFS($C$12:$C$183,"기능",$F$12:$F$183,"있음")</f>
         <v/>
       </c>
     </row>
@@ -4453,7 +4372,7 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>COUNTIFS($C$12:$C$186,"기능",$F$12:$F$186,"없음")</f>
+        <f>COUNTIFS($C$12:$C$183,"기능",$F$12:$F$183,"없음")</f>
         <v/>
       </c>
     </row>
@@ -4464,7 +4383,7 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>COUNTIF($C$12:$C$186,"불변규칙")</f>
+        <f>COUNTIF($C$12:$C$183,"불변규칙")</f>
         <v/>
       </c>
     </row>
@@ -4475,7 +4394,7 @@
         </is>
       </c>
       <c r="B9" s="8">
-        <f>COUNTIF($C$12:$C$186,"미구현")</f>
+        <f>COUNTIF($C$12:$C$183,"미구현")</f>
         <v/>
       </c>
     </row>
@@ -10619,7 +10538,7 @@
       </c>
       <c r="D181" s="9" t="inlineStr">
         <is>
-          <t>소프트웨어 개발보안 준수 — 부분 — 개별 조치는 있지만(§1-2 #2) 시큐어코딩 점검 기준표·점검 기록이 없다</t>
+          <t>이용자 매뉴얼 제작·게시판 탑재, 어플 사용 교육 자료 — 부분 — 관리자 웹 화면별 도움말과 회원 웹 이용 안내는 있다. 별도 사용자 매뉴얼(교육 자료 1편)과 게시판 탑재는 없다. 대면 교육은 해당 없음</t>
         </is>
       </c>
       <c r="E181" s="11" t="inlineStr">
@@ -10634,7 +10553,7 @@
       </c>
       <c r="G181" s="9" t="inlineStr">
         <is>
-          <t>설치및운영(1-2 #2)</t>
+          <t>과업4·산출물5(p.4·p.7)</t>
         </is>
       </c>
     </row>
@@ -10656,12 +10575,12 @@
       </c>
       <c r="D182" s="9" t="inlineStr">
         <is>
-          <t>보안관리계획(인원·문서·장비) — 없다. 개인정보처리방침은 회원 웹 초안으로 작성(D51)</t>
-        </is>
-      </c>
-      <c r="E182" s="12" t="inlineStr">
-        <is>
-          <t>미구현</t>
+          <t>단계별 개발 진행 보고서 5부 — 부분 — 진행 기록(docs/log/ 130여 건)·발표 자료는 있지만 개발·테스트·검수·도입·기대효과 단계별 보고서 형식은 없다</t>
+        </is>
+      </c>
+      <c r="E182" s="11" t="inlineStr">
+        <is>
+          <t>부분</t>
         </is>
       </c>
       <c r="F182" s="9" t="inlineStr">
@@ -10671,123 +10590,12 @@
       </c>
       <c r="G182" s="9" t="inlineStr">
         <is>
-          <t>보안요건(1-2 #8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="9" t="inlineStr">
-        <is>
-          <t>GAP-07</t>
-        </is>
-      </c>
-      <c r="B183" s="9" t="inlineStr">
-        <is>
-          <t>RFP 공통</t>
-        </is>
-      </c>
-      <c r="C183" s="9" t="inlineStr">
-        <is>
-          <t>미구현</t>
-        </is>
-      </c>
-      <c r="D183" s="9" t="inlineStr">
-        <is>
-          <t>지식재산권·저작권 점검 — 부분 — 오픈소스만 쓰지만 의존성 라이선스 목록·점검 기록이 없다</t>
-        </is>
-      </c>
-      <c r="E183" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
-        </is>
-      </c>
-      <c r="F183" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G183" s="9" t="inlineStr">
-        <is>
-          <t>규정의준수(1-2 #10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="9" t="inlineStr">
-        <is>
-          <t>GAP-08</t>
-        </is>
-      </c>
-      <c r="B184" s="9" t="inlineStr">
-        <is>
-          <t>RFP 공통</t>
-        </is>
-      </c>
-      <c r="C184" s="9" t="inlineStr">
-        <is>
-          <t>미구현</t>
-        </is>
-      </c>
-      <c r="D184" s="9" t="inlineStr">
-        <is>
-          <t>이용자 매뉴얼 제작·게시판 탑재, 어플 사용 교육 자료 — 부분 — 관리자 웹 화면별 도움말과 회원 웹 이용 안내는 있다. 별도 사용자 매뉴얼(교육 자료 1편)과 게시판 탑재는 없다. 대면 교육은 해당 없음</t>
-        </is>
-      </c>
-      <c r="E184" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
-        </is>
-      </c>
-      <c r="F184" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G184" s="9" t="inlineStr">
-        <is>
-          <t>과업4·산출물5(p.4·p.7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="9" t="inlineStr">
-        <is>
-          <t>GAP-09</t>
-        </is>
-      </c>
-      <c r="B185" s="9" t="inlineStr">
-        <is>
-          <t>RFP 공통</t>
-        </is>
-      </c>
-      <c r="C185" s="9" t="inlineStr">
-        <is>
-          <t>미구현</t>
-        </is>
-      </c>
-      <c r="D185" s="9" t="inlineStr">
-        <is>
-          <t>단계별 개발 진행 보고서 5부 — 부분 — 진행 기록(docs/log/ 130여 건)·발표 자료는 있지만 개발·테스트·검수·도입·기대효과 단계별 보고서 형식은 없다</t>
-        </is>
-      </c>
-      <c r="E185" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
-        </is>
-      </c>
-      <c r="F185" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G185" s="9" t="inlineStr">
-        <is>
           <t>산출물4(p.7)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A11:G185"/>
+  <autoFilter ref="A11:G182"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11322,7 +11130,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>1인 개발 구조상 "발주기관/전문가 검증" 주체가 없음 — CI(lint·빌드·jest·문서 검사)와 커밋 전 hook, 도메인 문서 §11 검증현황으로 대체. 개발보안은 개별 조치(비밀값 부팅 검사·1회용 갱신 토큰·응답 마스킹·지점 격리 가드·로그인 rate limit)만 있고 점검 기준표는 없음</t>
+          <t>1인 개발 구조상 "발주기관/전문가 검증" 주체가 없음 — CI(lint·빌드·jest·문서 검사)와 커밋 전 hook, 도메인 문서 §11 검증현황으로 대체. 개발보안은 행안부 구현단계 보안약점 49개로 점검했다(secure-coding-checklist — 대응 34·부분 4·해당 없음 11, 점검 중 찾은 문서 주소 XSS는 수정, log/139)</t>
         </is>
       </c>
     </row>
@@ -11484,7 +11292,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>개인정보처리방침을 회원 웹 화면(/m/privacy)으로 작성 — 수집 항목·열람 범위·보관·처리 위탁(26조: Supabase·AWS·Cloudflare). 시연용 초안, 가입 시 동의는 화면에서만 받음(D51). 보안관리계획(인원·문서·장비)은 없음</t>
+          <t>개인정보처리방침을 회원 웹 화면(/m/privacy)으로 작성 — 수집 항목·열람 범위·보관·처리 위탁(26조: Supabase·AWS·Cloudflare). 시연용 초안, 가입 시 동의는 화면에서만 받음(D51). 보안관리계획은 security-plan(인원·문서·장비·비밀값·위탁, 지금 약점 9건과 조치 계획 — log/139)</t>
         </is>
       </c>
     </row>
@@ -11538,7 +11346,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>오픈소스 라이선스(MIT/Apache 등) 패키지만 사용 — 별도 점검 문서는 없음</t>
+          <t>운영 의존성 219개가 모두 허용형 라이선스(MIT·ISC·Apache-2.0·BSD 등, copyleft 없음) — dependency-licenses를 scripts/license-report.mjs가 만들고 --check로 다시 점검(log/139). 이미지·아이콘은 자체 제작</t>
         </is>
       </c>
     </row>
@@ -11845,7 +11653,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -11855,22 +11663,22 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>12/19 = 63% / 95%</t>
+          <t>16/19 = 84% / 100%</t>
         </is>
       </c>
     </row>
@@ -11929,7 +11737,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>45</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -11939,12 +11747,12 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -11954,7 +11762,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>47/64 = 73% / 94%</t>
+          <t>51/64 = 80% / 95%</t>
         </is>
       </c>
     </row>
@@ -12898,14 +12706,14 @@
           <t>소프트웨어 개발보안 준수</t>
         </is>
       </c>
-      <c r="D49" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
+      <c r="D49" s="10" t="inlineStr">
+        <is>
+          <t>구현</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>개별 조치만, 점검 기준표 없음(§2-3)</t>
+          <t>행안부 구현단계 보안약점 49개 점검표(secure-coding-checklist — 대응 34·부분 4·해당 없음 11), 남은 조치 4건 표로 관리, 점검 중 찾은 XSS 수정(document-rules)</t>
         </is>
       </c>
     </row>
@@ -13357,14 +13165,14 @@
           <t>인원·문서·장비 보안관리계획 수립</t>
         </is>
       </c>
-      <c r="D66" s="12" t="inlineStr">
-        <is>
-          <t>미구현</t>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>구현</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
-          <t>문서 없음</t>
+          <t>security-plan — 인원·문서·장비·비밀값·운영 보호·위탁, 지금 약점 9건과 조치 계획</t>
         </is>
       </c>
     </row>
@@ -13391,7 +13199,7 @@
       </c>
       <c r="E67" s="4" t="inlineStr">
         <is>
-          <t>처리방침 초안의 위탁 고지(D51), 위탁 계약·점검은 없음</t>
+          <t>처리방침 초안의 위탁 고지(D51), 수탁자·업무·위치 표(security-plan §7). 위탁 계약 문서 보관·수탁자 감독 기록은 없음(실데이터 운영 전 조치)</t>
         </is>
       </c>
     </row>
@@ -13465,14 +13273,14 @@
           <t>산출물의 지식재산권 주의·준수</t>
         </is>
       </c>
-      <c r="D70" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
+      <c r="D70" s="10" t="inlineStr">
+        <is>
+          <t>구현</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
-          <t>오픈소스만 사용, 점검 기록 없음</t>
+          <t>운영 의존성 219개 라이선스 목록·허용형 점검(dependency-licenses, license-report.mjs --check)</t>
         </is>
       </c>
     </row>
@@ -13492,14 +13300,14 @@
           <t>저작권 문제가 없는 저작물 구현</t>
         </is>
       </c>
-      <c r="D71" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
+      <c r="D71" s="10" t="inlineStr">
+        <is>
+          <t>구현</t>
         </is>
       </c>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>같은 이유</t>
+          <t>같은 목록 + 이미지·아이콘 자체 제작, 외부 글꼴·이미지 파일 없음</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
공지 대상 시설 지정 — RFP F4-3(게시판 ADR-BRD-05, D28·D46, log/145)
- Post.facilityId(선택, Facility FK) + 같은 지점 트리거 post_facility_branch 마이그레이션
- 작성: @ScopedResource('facility', body)로 다른 지점 시설 403·없는 시설 404, 본사 공지 400
- 수정: 그 글 지점의 시설만(400 FACILITY_BRANCH_MISMATCH), null 해제. 목록 ?facilityId= 필터
- 관리자 웹 글쓰기·수정 "대상 시설", 회원 웹 공지 시설 고르기·표시
- post-facility.spec 5건, branch-isolation 공격 케이스, e2e admin-branch·member-notice 확장
- 추적표 F4-3 구현(80% → 81%), 요구사항·데이터 정의서 재생성(데이터 정의서 생성기 SupportRequest 누락 수정)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhHabvYheW2oxJWYuUifjJ
</commit_message>
<xml_diff>
--- a/docs/deliverables/요구사항정의서.xlsx
+++ b/docs/deliverables/요구사항정의서.xlsx
@@ -24,7 +24,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="범위 제외" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'요구사항 총괄'!$A$11:$G$182</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'요구사항 총괄'!$A$11:$G$181</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'RFP 충족 판정'!$A$17:$E$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -635,7 +635,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-19 저장소(dev 브랜치) — 도메인 문서·요구사항추적표·실제 API 라우트에서 자동 생성</t>
+          <t>2026-10-20 저장소(dev 브랜치) — 도메인 문서·요구사항추적표·실제 API 라우트에서 자동 생성</t>
         </is>
       </c>
     </row>
@@ -659,7 +659,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>도메인 9개 · 기능(API) 97개 · 불변규칙 26개 · RFP 미구현·부분 6건 · 자동 테스트 파일 43개</t>
+          <t>도메인 9개 · 기능(API) 97개 · 불변규칙 26개 · RFP 미구현·부분 5건 · 자동 테스트 파일 45개</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>조항 72개 중 해당 없음 8개를 뺀 충족률 51/64 = 80% / 95%(구현+조정 / 부분 포함)</t>
+          <t>조항 72개 중 해당 없음 8개를 뺀 충족률 52/64 = 81% / 95%(구현+조정 / 부분 포함)</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/예약및결제.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/예약및결제.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/강사프로그램게시.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/강사프로그램게시.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>
@@ -2489,7 +2489,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/혼잡도관리.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/혼잡도관리.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3059,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/자원문서관리.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/자원문서관리.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3949,17 +3949,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>게시판(1-1 #4)</t>
+          <t>시스템가용성(1-1 #10)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>현장→이용자 "각 시설에 대한" 공지 글·이미지</t>
+          <t>메모리 평균 85% 이하 유지</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>부분 — 공지는 지점 단위라 시설을 지정할 수 없다(이미지는 회원 웹 공지 상세 본문 아래에 보인다, log/137)</t>
+          <t>부분 — 경보 절차는 작성(aws-lambda/README §6). AWS 콘솔 적용은 사용자 작업 — 아직 없음</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -3976,17 +3976,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>시스템가용성(1-1 #10)</t>
+          <t>UI 보안(1-2 #7)</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>메모리 평균 85% 이하 유지</t>
+          <t>결제 시스템의 금융·보안기관 연계 가능 여부 확인</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>부분 — 경보 절차는 작성(aws-lambda/README §6). AWS 콘솔 적용은 사용자 작업 — 아직 없음</t>
+          <t>부분 — 모의 결제와 결제 어댑터 설계(ADR-RSV-03)만. PG사 연계 요건 확인 문서 없음</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
@@ -4003,17 +4003,17 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>UI 보안(1-2 #7)</t>
+          <t>과업4·산출물5(p.4·p.7)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>결제 시스템의 금융·보안기관 연계 가능 여부 확인</t>
+          <t>이용자 매뉴얼 제작·게시판 탑재, 어플 사용 교육 자료</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>부분 — 모의 결제와 결제 어댑터 설계(ADR-RSV-03)만. PG사 연계 요건 확인 문서 없음</t>
+          <t>부분 — 관리자 웹 화면별 도움말과 회원 웹 이용 안내는 있다. 별도 사용자 매뉴얼(교육 자료 1편)과 게시판 탑재는 없다. 대면 교육은 해당 없음</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
@@ -4030,17 +4030,17 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>과업4·산출물5(p.4·p.7)</t>
+          <t>산출물4(p.7)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>이용자 매뉴얼 제작·게시판 탑재, 어플 사용 교육 자료</t>
+          <t>단계별 개발 진행 보고서 5부</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>부분 — 관리자 웹 화면별 도움말과 회원 웹 이용 안내는 있다. 별도 사용자 매뉴얼(교육 자료 1편)과 게시판 탑재는 없다. 대면 교육은 해당 없음</t>
+          <t>부분 — 진행 기록(docs/log/ 130여 건)·발표 자료는 있지만 개발·테스트·검수·도입·기대효과 단계별 보고서 형식은 없다</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
@@ -4049,56 +4049,29 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>GAP-06</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>산출물4(p.7)</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>단계별 개발 진행 보고서 5부</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>부분 — 진행 기록(docs/log/ 130여 건)·발표 자료는 있지만 개발·테스트·검수·도입·기대효과 단계별 보고서 형식은 없다</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>API는 있고 화면이 없는 것</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="16" t="inlineStr">
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>지금은 없다(로컬 전용 dev-storage 경로 제외). 마지막 항목이던 관리자의 직원 업무일지 열람은 2026-10-14 직원 상세에 붙였다(D51, log/112).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>설계는 있지만 미구현인 도메인 규칙</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="16" t="inlineStr">
+    <row r="15" ht="36" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>결제 PaymentGateway 어댑터(ADR-RSV-03) — 실 PG를 붙일 때 필요하다.</t>
         </is>
@@ -4106,8 +4079,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A13:E13"/>
+    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4305,7 +4278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G182"/>
+  <dimension ref="A1:G181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4350,7 +4323,7 @@
         </is>
       </c>
       <c r="B5" s="8">
-        <f>COUNTIF($C$12:$C$183,"기능")</f>
+        <f>COUNTIF($C$12:$C$182,"기능")</f>
         <v/>
       </c>
     </row>
@@ -4361,7 +4334,7 @@
         </is>
       </c>
       <c r="B6" s="8">
-        <f>COUNTIFS($C$12:$C$183,"기능",$F$12:$F$183,"있음")</f>
+        <f>COUNTIFS($C$12:$C$182,"기능",$F$12:$F$182,"있음")</f>
         <v/>
       </c>
     </row>
@@ -4372,7 +4345,7 @@
         </is>
       </c>
       <c r="B7" s="8">
-        <f>COUNTIFS($C$12:$C$183,"기능",$F$12:$F$183,"없음")</f>
+        <f>COUNTIFS($C$12:$C$182,"기능",$F$12:$F$182,"없음")</f>
         <v/>
       </c>
     </row>
@@ -4383,7 +4356,7 @@
         </is>
       </c>
       <c r="B8" s="8">
-        <f>COUNTIF($C$12:$C$183,"불변규칙")</f>
+        <f>COUNTIF($C$12:$C$182,"불변규칙")</f>
         <v/>
       </c>
     </row>
@@ -4394,7 +4367,7 @@
         </is>
       </c>
       <c r="B9" s="8">
-        <f>COUNTIF($C$12:$C$183,"미구현")</f>
+        <f>COUNTIF($C$12:$C$182,"미구현")</f>
         <v/>
       </c>
     </row>
@@ -6723,7 +6696,7 @@
       </c>
       <c r="G75" s="4" t="inlineStr">
         <is>
-          <t>post-attachments·post-rules(동시 조회수·소프트 삭제·수정/삭제 권한·작성 범위)·posts-member-visibility·contract-termination·branch-isolation spec</t>
+          <t>post-facility·post-attachments·post-rules(동시 조회수·소프트 삭제·수정/삭제 권한·작성 범위)·posts-member-visibility·contract-termination·branch-isolation spec</t>
         </is>
       </c>
     </row>
@@ -6760,7 +6733,7 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>post-attachments·post-rules(동시 조회수·소프트 삭제·수정/삭제 권한·작성 범위)·posts-member-visibility·contract-termination·branch-isolation spec</t>
+          <t>post-facility·post-attachments·post-rules(동시 조회수·소프트 삭제·수정/삭제 권한·작성 범위)·posts-member-visibility·contract-termination·branch-isolation spec</t>
         </is>
       </c>
     </row>
@@ -10427,7 +10400,7 @@
       </c>
       <c r="D178" s="9" t="inlineStr">
         <is>
-          <t>현장→이용자 "각 시설에 대한" 공지 글·이미지 — 부분 — 공지는 지점 단위라 시설을 지정할 수 없다(이미지는 회원 웹 공지 상세 본문 아래에 보인다, log/137)</t>
+          <t>메모리 평균 85% 이하 유지 — 부분 — 경보 절차는 작성(aws-lambda/README §6). AWS 콘솔 적용은 사용자 작업 — 아직 없음</t>
         </is>
       </c>
       <c r="E178" s="11" t="inlineStr">
@@ -10442,7 +10415,7 @@
       </c>
       <c r="G178" s="9" t="inlineStr">
         <is>
-          <t>게시판(1-1 #4)</t>
+          <t>시스템가용성(1-1 #10)</t>
         </is>
       </c>
     </row>
@@ -10464,7 +10437,7 @@
       </c>
       <c r="D179" s="9" t="inlineStr">
         <is>
-          <t>메모리 평균 85% 이하 유지 — 부분 — 경보 절차는 작성(aws-lambda/README §6). AWS 콘솔 적용은 사용자 작업 — 아직 없음</t>
+          <t>결제 시스템의 금융·보안기관 연계 가능 여부 확인 — 부분 — 모의 결제와 결제 어댑터 설계(ADR-RSV-03)만. PG사 연계 요건 확인 문서 없음</t>
         </is>
       </c>
       <c r="E179" s="11" t="inlineStr">
@@ -10479,7 +10452,7 @@
       </c>
       <c r="G179" s="9" t="inlineStr">
         <is>
-          <t>시스템가용성(1-1 #10)</t>
+          <t>UI 보안(1-2 #7)</t>
         </is>
       </c>
     </row>
@@ -10501,7 +10474,7 @@
       </c>
       <c r="D180" s="9" t="inlineStr">
         <is>
-          <t>결제 시스템의 금융·보안기관 연계 가능 여부 확인 — 부분 — 모의 결제와 결제 어댑터 설계(ADR-RSV-03)만. PG사 연계 요건 확인 문서 없음</t>
+          <t>이용자 매뉴얼 제작·게시판 탑재, 어플 사용 교육 자료 — 부분 — 관리자 웹 화면별 도움말과 회원 웹 이용 안내는 있다. 별도 사용자 매뉴얼(교육 자료 1편)과 게시판 탑재는 없다. 대면 교육은 해당 없음</t>
         </is>
       </c>
       <c r="E180" s="11" t="inlineStr">
@@ -10516,7 +10489,7 @@
       </c>
       <c r="G180" s="9" t="inlineStr">
         <is>
-          <t>UI 보안(1-2 #7)</t>
+          <t>과업4·산출물5(p.4·p.7)</t>
         </is>
       </c>
     </row>
@@ -10538,7 +10511,7 @@
       </c>
       <c r="D181" s="9" t="inlineStr">
         <is>
-          <t>이용자 매뉴얼 제작·게시판 탑재, 어플 사용 교육 자료 — 부분 — 관리자 웹 화면별 도움말과 회원 웹 이용 안내는 있다. 별도 사용자 매뉴얼(교육 자료 1편)과 게시판 탑재는 없다. 대면 교육은 해당 없음</t>
+          <t>단계별 개발 진행 보고서 5부 — 부분 — 진행 기록(docs/log/ 130여 건)·발표 자료는 있지만 개발·테스트·검수·도입·기대효과 단계별 보고서 형식은 없다</t>
         </is>
       </c>
       <c r="E181" s="11" t="inlineStr">
@@ -10553,49 +10526,12 @@
       </c>
       <c r="G181" s="9" t="inlineStr">
         <is>
-          <t>과업4·산출물5(p.4·p.7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="9" t="inlineStr">
-        <is>
-          <t>GAP-06</t>
-        </is>
-      </c>
-      <c r="B182" s="9" t="inlineStr">
-        <is>
-          <t>RFP 공통</t>
-        </is>
-      </c>
-      <c r="C182" s="9" t="inlineStr">
-        <is>
-          <t>미구현</t>
-        </is>
-      </c>
-      <c r="D182" s="9" t="inlineStr">
-        <is>
-          <t>단계별 개발 진행 보고서 5부 — 부분 — 진행 기록(docs/log/ 130여 건)·발표 자료는 있지만 개발·테스트·검수·도입·기대효과 단계별 보고서 형식은 없다</t>
-        </is>
-      </c>
-      <c r="E182" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
-        </is>
-      </c>
-      <c r="F182" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G182" s="9" t="inlineStr">
-        <is>
           <t>산출물4(p.7)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A11:G182"/>
+  <autoFilter ref="A11:G181"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11611,7 +11547,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>23</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -11621,7 +11557,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -11636,7 +11572,7 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>25/28 = 89% / 100%</t>
+          <t>26/28 = 93% / 100%</t>
         </is>
       </c>
     </row>
@@ -11737,7 +11673,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>46</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -11747,7 +11683,7 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -11762,7 +11698,7 @@
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>51/64 = 80% / 95%</t>
+          <t>52/64 = 81% / 95%</t>
         </is>
       </c>
     </row>
@@ -12220,14 +12156,14 @@
           <t>현장→이용자 각 시설에 대한 공지 글·이미지 작성</t>
         </is>
       </c>
-      <c r="D31" s="11" t="inlineStr">
-        <is>
-          <t>부분</t>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>구현</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>지점 공지 글·이미지(회원 웹 본문 아래 표시, log/137)는 됨. 시설 지정 없음</t>
+          <t>지점 공지에 대상 시설 지정(게시판 ADR-BRD-05, log/145) — 관리자 웹 글쓰기·수정에서 선택, 회원 웹 시설로 거르기·표시. 이미지는 두 웹 모두 바로 표시(log/137·144)</t>
         </is>
       </c>
     </row>
@@ -13830,7 +13766,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/권한관리.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/권한관리.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>
@@ -14648,7 +14584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/인사정보관리.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/인사정보관리.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>
@@ -15682,7 +15618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -15703,7 +15639,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/근태관리.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/근태관리.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>
@@ -16562,8 +16498,28 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>ADR-ATT-05</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>겹치는 휴가 신청·승인 금지(직원 행 락, 연차 이중 차감 방지)</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="14" t="n"/>
+      <c r="E47" s="15" t="n"/>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>구현(log/141)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="B45:E45"/>
@@ -16575,6 +16531,7 @@
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B44:E44"/>
     <mergeCell ref="C15:F15"/>
+    <mergeCell ref="B47:E47"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="B8:F8"/>
     <mergeCell ref="B22:F22"/>
@@ -16591,7 +16548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -16612,7 +16569,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/게시판.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/게시판.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>
@@ -16841,7 +16798,7 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>post-attachments·post-rules(동시 조회수·소프트 삭제·수정/삭제 권한·작성 범위)·posts-member-visibility·contract-termination·branch-isolation spec</t>
+          <t>post-facility·post-attachments·post-rules(동시 조회수·소프트 삭제·수정/삭제 권한·작성 범위)·posts-member-visibility·contract-termination·branch-isolation spec</t>
         </is>
       </c>
     </row>
@@ -17275,31 +17232,51 @@
       <c r="E39" s="15" t="n"/>
       <c r="F39" s="10" t="inlineStr">
         <is>
-          <t>구현(log/121, 배포 저장소 설정 전)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+          <t>구현(log/121), 배포 실제 파일 확인(log/144)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>ADR-BRD-05</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>지점 공지의 대상 시설(Post.facilityId, 선택) — 다른 지점 시설 403, 본사 공지 400, 목록 facilityId 필터</t>
+        </is>
+      </c>
+      <c r="C40" s="14" t="n"/>
+      <c r="D40" s="14" t="n"/>
+      <c r="E40" s="15" t="n"/>
+      <c r="F40" s="10" t="inlineStr">
+        <is>
+          <t>구현(log/145, 배포 DB 적용 대기)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>미구현·범위 제외(도메인 문서 기준)</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="30" customHeight="1">
-      <c r="A42" s="16" t="inlineStr">
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="16" t="inlineStr">
         <is>
           <t>pinned·읽음 확인(범위 제외), category 필터 UI, TrainingLog</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="C13:F13"/>
     <mergeCell ref="B36:E36"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B7:F7"/>
-    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="B40:E40"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="B20:F20"/>
     <mergeCell ref="B37:E37"/>
@@ -17310,6 +17287,7 @@
     <mergeCell ref="C11:F11"/>
     <mergeCell ref="B19:E19"/>
     <mergeCell ref="C14:F14"/>
+    <mergeCell ref="A43:F43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -17342,7 +17320,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>원천: docs/domains/회원관리.md · 기능 명세는 코드 실측(2026-10-19 저장소 기준)</t>
+          <t>원천: docs/domains/회원관리.md · 기능 명세는 코드 실측(2026-10-20 저장소 기준)</t>
         </is>
       </c>
     </row>

</xml_diff>